<commit_message>
Update Gold Master files for scenario10
- Update expected output files for scenario10
- Gold Master test data updated with correct expected results
</commit_message>
<xml_diff>
--- a/doctool/test/auto/scenario10/システム機能設計書_サンプル_S10_expected.xlsx
+++ b/doctool/test/auto/scenario10/システム機能設計書_サンプル_S10_expected.xlsx
@@ -5,39 +5,37 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tie303229\AppData\Local\Temp\pytest-of-tie303229\pytest-21\scenario09_0\scenario09\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PJ\01.Nablarch\repo\review-support-tool\doctool\test\auto\scenario10\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FA0F477-3786-4A8A-96DC-D33FA1D52AF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA9AC98A-DA7F-4DD7-B01B-2E1FF5314191}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="3120" windowWidth="38700" windowHeight="15345" tabRatio="822" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1560" yWindow="4965" windowWidth="24285" windowHeight="13710" tabRatio="822" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="レビュー結果1回目" sheetId="9" r:id="rId1"/>
-    <sheet name="表紙" sheetId="1" r:id="rId2"/>
-    <sheet name="変更履歴" sheetId="2" r:id="rId3"/>
-    <sheet name="目次" sheetId="3" r:id="rId4"/>
-    <sheet name="1.  画面取引定義" sheetId="4" r:id="rId5"/>
-    <sheet name="2. WA1020101(プロジェクト登録画面)" sheetId="5" r:id="rId6"/>
-    <sheet name="3. WA1020102(プロジェクト登録確認画面)" sheetId="6" r:id="rId7"/>
-    <sheet name="4. WA1020103(プロジェクト登録完了画面)" sheetId="7" r:id="rId8"/>
-    <sheet name="データ" sheetId="8" state="hidden" r:id="rId9"/>
+    <sheet name="表紙" sheetId="1" r:id="rId1"/>
+    <sheet name="変更履歴" sheetId="2" r:id="rId2"/>
+    <sheet name="目次" sheetId="3" r:id="rId3"/>
+    <sheet name="1.  画面取引定義" sheetId="4" r:id="rId4"/>
+    <sheet name="2. WA1020101(プロジェクト登録画面)" sheetId="5" r:id="rId5"/>
+    <sheet name="3. WA1020102(プロジェクト登録確認画面)" sheetId="6" r:id="rId6"/>
+    <sheet name="4. WA1020103(プロジェクト登録完了画面)" sheetId="7" r:id="rId7"/>
+    <sheet name="データ" sheetId="8" state="hidden" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_Toc46209822" localSheetId="4">'1.  画面取引定義'!$B$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="4">'1.  画面取引定義'!$A$1:$AI$21</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="5">'2. WA1020101(プロジェクト登録画面)'!$A$1:$AI$180</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="6">'3. WA1020102(プロジェクト登録確認画面)'!$A$1:$AI$136</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="7">'4. WA1020103(プロジェクト登録完了画面)'!$A$1:$AI$68</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="8">データ!$A$1:$E$15</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">レビュー結果1回目!$A$1:$K$18</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">表紙!$A$1:$S$39</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">変更履歴!$A$1:$AI$34</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">目次!$A$1:$AI$33</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="4">'1.  画面取引定義'!$1:$4</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="5">'2. WA1020101(プロジェクト登録画面)'!$1:$4</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="6">'3. WA1020102(プロジェクト登録確認画面)'!$1:$4</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="7">'4. WA1020103(プロジェクト登録完了画面)'!$1:$4</definedName>
+    <definedName name="_Toc46209822" localSheetId="3">'1.  画面取引定義'!$B$5</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'1.  画面取引定義'!$A$1:$AI$21</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'2. WA1020101(プロジェクト登録画面)'!$A$1:$AI$180</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">'3. WA1020102(プロジェクト登録確認画面)'!$A$1:$AI$136</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="6">'4. WA1020103(プロジェクト登録完了画面)'!$A$1:$AI$68</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="7">データ!$A$1:$E$15</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">表紙!$A$1:$S$39</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">変更履歴!$A$1:$AI$34</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">目次!$A$1:$AI$33</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'1.  画面取引定義'!$1:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'2. WA1020101(プロジェクト登録画面)'!$1:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'3. WA1020102(プロジェクト登録確認画面)'!$1:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">'4. WA1020103(プロジェクト登録完了画面)'!$1:$4</definedName>
     <definedName name="引継項目格納先">データ!$B$2:$B$2</definedName>
     <definedName name="画面項目種類">データ!$A$2:$A$14</definedName>
     <definedName name="種別一覧">データ!$C$2:$C$7</definedName>
@@ -65,73 +63,6 @@
     <author>作成者</author>
   </authors>
   <commentList>
-    <comment ref="A4" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000001000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="ＭＳ 明朝"/>
-            <family val="1"/>
-            <charset val="128"/>
-          </rPr>
-          <t>山田　太郎:*
-実施日:2023/08/01
-開始:09:00
-終了:14:00
-レビュー時間:200</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000002000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="ＭＳ 明朝"/>
-            <family val="1"/>
-            <charset val="128"/>
-          </rPr>
-          <t>山田　太郎:a
-レビュー指摘コメントの例。
-自動で挿入される名前とコロンの直後に指摘分類をa～iで書く。
-※レビュー日時を書く場合はコロンの直後に*を書く。</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E60" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000003000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="ＭＳ 明朝"/>
-            <family val="1"/>
-            <charset val="128"/>
-          </rPr>
-          <t>山田　太郎:b
-対応内容の例。
----
-対応内容はデリミタ（---）の後に記入する。</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E62" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000004000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="ＭＳ 明朝"/>
-            <family val="1"/>
-            <charset val="128"/>
-          </rPr>
-          <t>山田　太郎:c
-対応内容を確認し、指摘をクローズする例。
----
-最後の行に「済」と書くと指摘をクローズできる。
-「済」の前にスペースを空けて確認日と確認者を書くこともできる。
-08/02山田 済</t>
-        </r>
-      </text>
-    </comment>
     <comment ref="A71" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000005000000}">
       <text>
         <r>
@@ -151,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="844" uniqueCount="319">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="773" uniqueCount="265">
   <si>
     <t>第１．２版</t>
   </si>
@@ -965,315 +896,16 @@
   <si>
     <t>file</t>
   </si>
-  <si>
-    <t>＜レビュー結果＞</t>
-    <rPh sb="5" eb="7">
-      <t>ケッカ</t>
-    </rPh>
-    <phoneticPr fontId="13"/>
-  </si>
-  <si>
-    <t>この列は削除しないでください。（行の高さ調整用です。）</t>
-    <rPh sb="2" eb="3">
-      <t>レツ</t>
-    </rPh>
-    <rPh sb="4" eb="6">
-      <t>サクジョ</t>
-    </rPh>
-    <rPh sb="16" eb="17">
-      <t>ギョウ</t>
-    </rPh>
-    <rPh sb="18" eb="19">
-      <t>タカ</t>
-    </rPh>
-    <rPh sb="20" eb="22">
-      <t>チョウセイ</t>
-    </rPh>
-    <rPh sb="22" eb="23">
-      <t>ヨウ</t>
-    </rPh>
-    <phoneticPr fontId="13"/>
-  </si>
-  <si>
-    <t>文書ID:</t>
-    <rPh sb="0" eb="2">
-      <t>ブンショ</t>
-    </rPh>
-    <phoneticPr fontId="13"/>
-  </si>
-  <si>
-    <t>レビュー日時</t>
-    <rPh sb="4" eb="6">
-      <t>ニチジ</t>
-    </rPh>
-    <phoneticPr fontId="13"/>
-  </si>
-  <si>
-    <t>対象ファイル</t>
-    <rPh sb="0" eb="2">
-      <t>タイショウ</t>
-    </rPh>
-    <phoneticPr fontId="13"/>
-  </si>
-  <si>
-    <t>回</t>
-    <rPh sb="0" eb="1">
-      <t>カイ</t>
-    </rPh>
-    <phoneticPr fontId="13"/>
-  </si>
-  <si>
-    <t>実施日</t>
-    <rPh sb="0" eb="3">
-      <t>ジッシビ</t>
-    </rPh>
-    <phoneticPr fontId="13"/>
-  </si>
-  <si>
-    <t>開始</t>
-    <rPh sb="0" eb="2">
-      <t>カイシ</t>
-    </rPh>
-    <phoneticPr fontId="13"/>
-  </si>
-  <si>
-    <t>終了</t>
-    <rPh sb="0" eb="2">
-      <t>シュウリョウ</t>
-    </rPh>
-    <phoneticPr fontId="13"/>
-  </si>
-  <si>
-    <t>レビュー時間</t>
-    <rPh sb="4" eb="6">
-      <t>ジカン</t>
-    </rPh>
-    <phoneticPr fontId="13"/>
-  </si>
-  <si>
-    <t>～</t>
-    <phoneticPr fontId="13"/>
-  </si>
-  <si>
-    <t>指摘件数</t>
-    <rPh sb="0" eb="2">
-      <t>シテキ</t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t>ケンスウ</t>
-    </rPh>
-    <phoneticPr fontId="13"/>
-  </si>
-  <si>
-    <t>a</t>
-    <phoneticPr fontId="13"/>
-  </si>
-  <si>
-    <t>b</t>
-    <phoneticPr fontId="13"/>
-  </si>
-  <si>
-    <t>c</t>
-    <phoneticPr fontId="13"/>
-  </si>
-  <si>
-    <t>d</t>
-    <phoneticPr fontId="13"/>
-  </si>
-  <si>
-    <t>e</t>
-    <phoneticPr fontId="13"/>
-  </si>
-  <si>
-    <t>f</t>
-    <phoneticPr fontId="13"/>
-  </si>
-  <si>
-    <t>g</t>
-    <phoneticPr fontId="13"/>
-  </si>
-  <si>
-    <t>h</t>
-    <phoneticPr fontId="13"/>
-  </si>
-  <si>
-    <t>i</t>
-    <phoneticPr fontId="13"/>
-  </si>
-  <si>
-    <t>対応状況</t>
-    <rPh sb="0" eb="2">
-      <t>タイオウ</t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t>ジョウキョウ</t>
-    </rPh>
-    <phoneticPr fontId="13"/>
-  </si>
-  <si>
-    <t>01_要件漏れ</t>
-  </si>
-  <si>
-    <t>02_要件誤り</t>
-  </si>
-  <si>
-    <t>11_機能・仕様漏れ</t>
-  </si>
-  <si>
-    <t>12_機能・仕様誤り</t>
-  </si>
-  <si>
-    <t>21_設計・ドキュメント規約違反</t>
-  </si>
-  <si>
-    <t>22_記述誤り</t>
-  </si>
-  <si>
-    <t>91_疑問点、確認</t>
-  </si>
-  <si>
-    <t>92_改善要望</t>
-  </si>
-  <si>
-    <t>93_仕様変更</t>
-  </si>
-  <si>
-    <t>計</t>
-    <rPh sb="0" eb="1">
-      <t>ケイ</t>
-    </rPh>
-    <phoneticPr fontId="13"/>
-  </si>
-  <si>
-    <t>済</t>
-    <rPh sb="0" eb="1">
-      <t>スミ</t>
-    </rPh>
-    <phoneticPr fontId="13"/>
-  </si>
-  <si>
-    <t>未</t>
-    <rPh sb="0" eb="1">
-      <t>ミ</t>
-    </rPh>
-    <phoneticPr fontId="13"/>
-  </si>
-  <si>
-    <t>指摘詳細</t>
-    <rPh sb="0" eb="2">
-      <t>シテキ</t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t>ショウサイ</t>
-    </rPh>
-    <phoneticPr fontId="13"/>
-  </si>
-  <si>
-    <t>集計用ワーク</t>
-    <rPh sb="0" eb="3">
-      <t>シュウケイヨウ</t>
-    </rPh>
-    <phoneticPr fontId="13"/>
-  </si>
-  <si>
-    <t>シート</t>
-    <phoneticPr fontId="13"/>
-  </si>
-  <si>
-    <t>場所</t>
-    <rPh sb="0" eb="2">
-      <t>バショ</t>
-    </rPh>
-    <phoneticPr fontId="13"/>
-  </si>
-  <si>
-    <t>指摘者</t>
-    <rPh sb="0" eb="2">
-      <t>シテキ</t>
-    </rPh>
-    <rPh sb="2" eb="3">
-      <t>シャ</t>
-    </rPh>
-    <phoneticPr fontId="13"/>
-  </si>
-  <si>
-    <t>指摘種別</t>
-    <rPh sb="0" eb="2">
-      <t>シテキ</t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t>シュベツ</t>
-    </rPh>
-    <phoneticPr fontId="13"/>
-  </si>
-  <si>
-    <t>指摘内容</t>
-    <rPh sb="0" eb="2">
-      <t>シテキ</t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t>ナイヨウ</t>
-    </rPh>
-    <phoneticPr fontId="13"/>
-  </si>
-  <si>
-    <t>システム機能設計書_サンプル_S09</t>
-  </si>
-  <si>
-    <t>B5</t>
-  </si>
-  <si>
-    <t>山田　太郎</t>
-  </si>
-  <si>
-    <t>a</t>
-  </si>
-  <si>
-    <t>レビュー指摘コメントの例。
-自動で挿入される名前とコロンの直後に指摘分類をa～iで書く。
-※レビュー日時を書く場合はコロンの直後に*を書く。</t>
-  </si>
-  <si>
-    <t>未</t>
-  </si>
-  <si>
-    <t>E60</t>
-  </si>
-  <si>
-    <t>b</t>
-  </si>
-  <si>
-    <t>対応内容の例。
----
-対応内容はデリミタ（---）の後に記入する。</t>
-  </si>
-  <si>
-    <t>E62</t>
-  </si>
-  <si>
-    <t>c</t>
-  </si>
-  <si>
-    <t>対応内容を確認し、指摘をクローズする例。
----
-最後の行に「済」と書くと指摘をクローズできる。
-「済」の前にスペースを空けて確認日と確認者を書くこともできる。
-08/02山田 済</t>
-  </si>
-  <si>
-    <t>済</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="176" formatCode="&quot;第&quot;0.00&quot;版&quot;"/>
     <numFmt numFmtId="177" formatCode="yyyy/mm/dd"/>
-    <numFmt numFmtId="178" formatCode="#"/>
   </numFmts>
-  <fonts count="27" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="9"/>
       <name val="ＭＳ 明朝"/>
@@ -1355,12 +987,6 @@
       <charset val="128"/>
     </font>
     <font>
-      <sz val="6"/>
-      <name val="ＭＳ Ｐゴシック"/>
-      <family val="3"/>
-      <charset val="128"/>
-    </font>
-    <font>
       <sz val="11"/>
       <name val="ＭＳ Ｐゴシック"/>
       <family val="3"/>
@@ -1415,42 +1041,8 @@
       <family val="1"/>
       <charset val="128"/>
     </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="ＭＳ Ｐゴシック"/>
-      <family val="3"/>
-      <charset val="128"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color indexed="9"/>
-      <name val="ＭＳ Ｐゴシック"/>
-      <family val="3"/>
-      <charset val="128"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color indexed="10"/>
-      <name val="ＭＳ Ｐゴシック"/>
-      <family val="3"/>
-      <charset val="128"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="MS UI Gothic"/>
-      <family val="3"/>
-      <charset val="128"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="MS UI Gothic"/>
-      <family val="3"/>
-      <charset val="128"/>
-    </font>
   </fonts>
-  <fills count="12">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1490,30 +1082,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.14999847407452621"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="42"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="26"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="43"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="47"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1969,21 +1537,21 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0">
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="9" fontId="12" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="299">
+  <cellXfs count="261">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2046,22 +1614,22 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2199,7 +1767,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
@@ -2332,8 +1900,8 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2414,7 +1982,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2484,7 +2052,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2628,121 +2196,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="11" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="11">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="11" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="11" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" xfId="11" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="2" xfId="11" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="3" xfId="11" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="10" xfId="11" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="10" xfId="11" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="10" xfId="11" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="11" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="11" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="14" fillId="0" borderId="10" xfId="11" applyNumberFormat="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="14" fillId="0" borderId="10" xfId="11" applyNumberFormat="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="11" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="10" xfId="11" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="8" borderId="10" xfId="11" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="8" borderId="10" xfId="11" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="8" borderId="10" xfId="11" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="8" borderId="0" xfId="11" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="178" fontId="14" fillId="0" borderId="10" xfId="11" applyNumberFormat="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="22" fillId="9" borderId="10" xfId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="8" borderId="10" xfId="11" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="22" fillId="9" borderId="10" xfId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="178" fontId="22" fillId="0" borderId="0" xfId="11" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="11" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="10" xfId="11" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="1" xfId="11" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="2" xfId="11" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="2" xfId="11" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="3" xfId="11" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="10" xfId="11" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" xfId="11" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="5">
-      <alignment vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="11" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="12">
@@ -2759,14 +2212,7 @@
     <cellStyle name="標準_画面標準" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="標準_画面標準定義" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
   </cellStyles>
-  <dxfs count="3">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor indexed="22"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <font>
         <b/>
@@ -2787,8 +2233,8 @@
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="MySqlDefault" pivot="0" table="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" dxfId="2"/>
-      <tableStyleElement type="headerRow" dxfId="1"/>
+      <tableStyleElement type="wholeTable" dxfId="1"/>
+      <tableStyleElement type="headerRow" dxfId="0"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -3179,693 +2625,6 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60953CFA-4394-4A9A-B107-E54DE2F94C40}">
-  <sheetPr codeName="SheetTemplate">
-    <tabColor indexed="44"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:U18"/>
-  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
-  <cols>
-    <col min="1" max="1" width="9.33203125" style="262"/>
-    <col min="2" max="11" width="17.6640625" style="262" customWidth="1"/>
-    <col min="12" max="20" width="4.5" style="262" customWidth="1"/>
-    <col min="21" max="21" width="98.1640625" style="262" customWidth="1"/>
-    <col min="22" max="16384" width="9.33203125" style="262"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.15">
-      <c r="A1" s="261" t="s">
-        <v>265</v>
-      </c>
-      <c r="L1" s="263"/>
-      <c r="U1" s="264" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.15">
-      <c r="A2" s="262" t="s">
-        <v>267</v>
-      </c>
-      <c r="E2" s="265" t="s">
-        <v>268</v>
-      </c>
-      <c r="F2" s="266"/>
-      <c r="G2" s="266"/>
-      <c r="H2" s="266"/>
-      <c r="I2" s="267"/>
-      <c r="L2" s="263"/>
-    </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.15">
-      <c r="A3" s="268" t="s">
-        <v>269</v>
-      </c>
-      <c r="B3" s="268"/>
-      <c r="C3" s="269" t="s">
-        <v>270</v>
-      </c>
-      <c r="E3" s="269" t="s">
-        <v>271</v>
-      </c>
-      <c r="F3" s="269" t="s">
-        <v>272</v>
-      </c>
-      <c r="G3" s="270"/>
-      <c r="H3" s="269" t="s">
-        <v>273</v>
-      </c>
-      <c r="I3" s="269" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.15">
-      <c r="A4" s="271" t="s">
-        <v>306</v>
-      </c>
-      <c r="B4" s="271"/>
-      <c r="C4" s="272">
-        <v>1</v>
-      </c>
-      <c r="E4" s="273">
-        <v>45139</v>
-      </c>
-      <c r="F4" s="274">
-        <v>0.375</v>
-      </c>
-      <c r="G4" s="275" t="s">
-        <v>275</v>
-      </c>
-      <c r="H4" s="274">
-        <v>0.58333333333333337</v>
-      </c>
-      <c r="I4" s="272">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.15">
-      <c r="A6" s="261" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.15">
-      <c r="B7" s="276" t="s">
-        <v>277</v>
-      </c>
-      <c r="C7" s="276" t="s">
-        <v>278</v>
-      </c>
-      <c r="D7" s="270" t="s">
-        <v>279</v>
-      </c>
-      <c r="E7" s="270" t="s">
-        <v>280</v>
-      </c>
-      <c r="F7" s="270" t="s">
-        <v>281</v>
-      </c>
-      <c r="G7" s="270" t="s">
-        <v>282</v>
-      </c>
-      <c r="H7" s="270" t="s">
-        <v>283</v>
-      </c>
-      <c r="I7" s="270" t="s">
-        <v>284</v>
-      </c>
-      <c r="J7" s="270" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="8" spans="1:21" ht="27" x14ac:dyDescent="0.15">
-      <c r="A8" s="269" t="s">
-        <v>286</v>
-      </c>
-      <c r="B8" s="277" t="s">
-        <v>287</v>
-      </c>
-      <c r="C8" s="277" t="s">
-        <v>288</v>
-      </c>
-      <c r="D8" s="277" t="s">
-        <v>289</v>
-      </c>
-      <c r="E8" s="278" t="s">
-        <v>290</v>
-      </c>
-      <c r="F8" s="277" t="s">
-        <v>291</v>
-      </c>
-      <c r="G8" s="277" t="s">
-        <v>292</v>
-      </c>
-      <c r="H8" s="277" t="s">
-        <v>293</v>
-      </c>
-      <c r="I8" s="277" t="s">
-        <v>294</v>
-      </c>
-      <c r="J8" s="278" t="s">
-        <v>295</v>
-      </c>
-      <c r="K8" s="279" t="s">
-        <v>296</v>
-      </c>
-      <c r="L8" s="280"/>
-      <c r="M8" s="280"/>
-      <c r="N8" s="280"/>
-      <c r="O8" s="280"/>
-      <c r="P8" s="280"/>
-      <c r="Q8" s="280"/>
-      <c r="R8" s="280"/>
-      <c r="S8" s="280"/>
-      <c r="T8" s="280"/>
-    </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.15">
-      <c r="A9" s="269" t="s">
-        <v>297</v>
-      </c>
-      <c r="B9" s="281" t="str">
-        <f>IF(SUMIF($K15:$K18,$A9,L15:L18)=0,"",SUMIF($K15:$K18,$A9,L15:L18))</f>
-        <v/>
-      </c>
-      <c r="C9" s="281" t="str">
-        <f>IF(SUMIF($K15:$K18,$A9,M15:M18)=0,"",SUMIF($K15:$K18,$A9,M15:M18))</f>
-        <v/>
-      </c>
-      <c r="D9" s="281">
-        <f>IF(SUMIF($K15:$K18,$A9,N15:N18)=0,"",SUMIF($K15:$K18,$A9,N15:N18))</f>
-        <v>1</v>
-      </c>
-      <c r="E9" s="281" t="str">
-        <f>IF(SUMIF($K15:$K18,$A9,O15:O18)=0,"",SUMIF($K15:$K18,$A9,O15:O18))</f>
-        <v/>
-      </c>
-      <c r="F9" s="281" t="str">
-        <f>IF(SUMIF($K15:$K18,$A9,P15:P18)=0,"",SUMIF($K15:$K18,$A9,P15:P18))</f>
-        <v/>
-      </c>
-      <c r="G9" s="281" t="str">
-        <f>IF(SUMIF($K15:$K18,$A9,Q15:Q18)=0,"",SUMIF($K15:$K18,$A9,Q15:Q18))</f>
-        <v/>
-      </c>
-      <c r="H9" s="281" t="str">
-        <f>IF(SUMIF($K15:$K18,$A9,R15:R18)=0,"",SUMIF($K15:$K18,$A9,R15:R18))</f>
-        <v/>
-      </c>
-      <c r="I9" s="281" t="str">
-        <f>IF(SUMIF($K15:$K18,$A9,S15:S18)=0,"",SUMIF($K15:$K18,$A9,S15:S18))</f>
-        <v/>
-      </c>
-      <c r="J9" s="281" t="str">
-        <f>IF(SUMIF($K15:$K18,$A9,T15:T18)=0,"",SUMIF($K15:$K18,$A9,T15:T18))</f>
-        <v/>
-      </c>
-      <c r="K9" s="282">
-        <f>SUM(B9:J9)</f>
-        <v>1</v>
-      </c>
-      <c r="L9" s="261"/>
-      <c r="M9" s="261"/>
-      <c r="N9" s="261"/>
-      <c r="O9" s="261"/>
-      <c r="P9" s="261"/>
-      <c r="Q9" s="261"/>
-      <c r="R9" s="261"/>
-      <c r="S9" s="261"/>
-      <c r="T9" s="261"/>
-    </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.15">
-      <c r="A10" s="269" t="s">
-        <v>298</v>
-      </c>
-      <c r="B10" s="281">
-        <f>IF(SUMIF($K15:$K18,$A10,L15:L18)=0,"",SUMIF($K15:$K18,$A10,L15:L18))</f>
-        <v>1</v>
-      </c>
-      <c r="C10" s="281">
-        <f>IF(SUMIF($K15:$K18,$A10,M15:M18)=0,"",SUMIF($K15:$K18,$A10,M15:M18))</f>
-        <v>1</v>
-      </c>
-      <c r="D10" s="281" t="str">
-        <f>IF(SUMIF($K15:$K18,$A10,N15:N18)=0,"",SUMIF($K15:$K18,$A10,N15:N18))</f>
-        <v/>
-      </c>
-      <c r="E10" s="281" t="str">
-        <f>IF(SUMIF($K15:$K18,$A10,O15:O18)=0,"",SUMIF($K15:$K18,$A10,O15:O18))</f>
-        <v/>
-      </c>
-      <c r="F10" s="281" t="str">
-        <f>IF(SUMIF($K15:$K18,$A10,P15:P18)=0,"",SUMIF($K15:$K18,$A10,P15:P18))</f>
-        <v/>
-      </c>
-      <c r="G10" s="281" t="str">
-        <f>IF(SUMIF($K15:$K18,$A10,Q15:Q18)=0,"",SUMIF($K15:$K18,$A10,Q15:Q18))</f>
-        <v/>
-      </c>
-      <c r="H10" s="281" t="str">
-        <f>IF(SUMIF($K15:$K18,$A10,R15:R18)=0,"",SUMIF($K15:$K18,$A10,R15:R18))</f>
-        <v/>
-      </c>
-      <c r="I10" s="281" t="str">
-        <f>IF(SUMIF($K15:$K18,$A10,S15:S18)=0,"",SUMIF($K15:$K18,$A10,S15:S18))</f>
-        <v/>
-      </c>
-      <c r="J10" s="281" t="str">
-        <f>IF(SUMIF($K15:$K18,$A10,T15:T18)=0,"",SUMIF($K15:$K18,$A10,T15:T18))</f>
-        <v/>
-      </c>
-      <c r="K10" s="282">
-        <f>SUM(B10:J10)</f>
-        <v>2</v>
-      </c>
-      <c r="L10" s="261"/>
-      <c r="M10" s="261"/>
-      <c r="N10" s="261"/>
-      <c r="O10" s="261"/>
-      <c r="P10" s="261"/>
-      <c r="Q10" s="261"/>
-      <c r="R10" s="261"/>
-      <c r="S10" s="261"/>
-      <c r="T10" s="261"/>
-    </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.15">
-      <c r="A11" s="283" t="s">
-        <v>296</v>
-      </c>
-      <c r="B11" s="284">
-        <f>SUM(B9:B10)</f>
-        <v>1</v>
-      </c>
-      <c r="C11" s="284">
-        <f t="shared" ref="C11:K11" si="0">SUM(C9:C10)</f>
-        <v>1</v>
-      </c>
-      <c r="D11" s="284">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="E11" s="284">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F11" s="284">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G11" s="284">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H11" s="284">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I11" s="284">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="J11" s="284">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="K11" s="284">
-        <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.15">
-      <c r="A12" s="261"/>
-      <c r="B12" s="285"/>
-      <c r="C12" s="285"/>
-      <c r="D12" s="285"/>
-      <c r="E12" s="285"/>
-      <c r="F12" s="285"/>
-      <c r="G12" s="285"/>
-      <c r="H12" s="285"/>
-      <c r="I12" s="285"/>
-      <c r="J12" s="285"/>
-      <c r="K12" s="285"/>
-    </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.15">
-      <c r="A13" s="286" t="s">
-        <v>299</v>
-      </c>
-      <c r="B13" s="287"/>
-      <c r="C13" s="287"/>
-      <c r="D13" s="287"/>
-      <c r="F13" s="287"/>
-      <c r="L13" s="263" t="s">
-        <v>300</v>
-      </c>
-      <c r="M13" s="263"/>
-      <c r="N13" s="263"/>
-      <c r="O13" s="263"/>
-      <c r="P13" s="263"/>
-      <c r="Q13" s="263"/>
-      <c r="R13" s="263"/>
-      <c r="S13" s="263"/>
-      <c r="T13" s="263"/>
-    </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.15">
-      <c r="A14" s="288" t="s">
-        <v>301</v>
-      </c>
-      <c r="B14" s="288" t="s">
-        <v>302</v>
-      </c>
-      <c r="C14" s="288" t="s">
-        <v>303</v>
-      </c>
-      <c r="D14" s="288" t="s">
-        <v>304</v>
-      </c>
-      <c r="E14" s="289" t="s">
-        <v>305</v>
-      </c>
-      <c r="F14" s="290"/>
-      <c r="G14" s="291"/>
-      <c r="H14" s="291"/>
-      <c r="I14" s="291"/>
-      <c r="J14" s="292"/>
-      <c r="K14" s="293" t="s">
-        <v>286</v>
-      </c>
-      <c r="L14" s="294" t="s">
-        <v>277</v>
-      </c>
-      <c r="M14" s="294" t="s">
-        <v>278</v>
-      </c>
-      <c r="N14" s="294" t="s">
-        <v>279</v>
-      </c>
-      <c r="O14" s="294" t="s">
-        <v>280</v>
-      </c>
-      <c r="P14" s="294" t="s">
-        <v>281</v>
-      </c>
-      <c r="Q14" s="294" t="s">
-        <v>282</v>
-      </c>
-      <c r="R14" s="294" t="s">
-        <v>283</v>
-      </c>
-      <c r="S14" s="294" t="s">
-        <v>284</v>
-      </c>
-      <c r="T14" s="294" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="15" spans="1:21" ht="40.5" x14ac:dyDescent="0.15">
-      <c r="A15" s="272" t="s">
-        <v>38</v>
-      </c>
-      <c r="B15" s="297" t="s">
-        <v>307</v>
-      </c>
-      <c r="C15" s="272" t="s">
-        <v>308</v>
-      </c>
-      <c r="D15" s="272" t="s">
-        <v>309</v>
-      </c>
-      <c r="E15" s="298" t="s">
-        <v>310</v>
-      </c>
-      <c r="F15" s="271"/>
-      <c r="G15" s="271"/>
-      <c r="H15" s="271"/>
-      <c r="I15" s="271"/>
-      <c r="J15" s="271"/>
-      <c r="K15" s="272" t="s">
-        <v>311</v>
-      </c>
-      <c r="L15" s="295">
-        <f t="shared" ref="L15:T18" si="1">IF($D15=L$14,1,0)</f>
-        <v>1</v>
-      </c>
-      <c r="M15" s="295">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="N15" s="295">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="O15" s="295">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="P15" s="295">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Q15" s="295">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R15" s="295">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="S15" s="295">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="T15" s="295">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="U15" s="296" t="str">
-        <f>IF(E15&lt;&gt;"",E15,"")</f>
-        <v>レビュー指摘コメントの例。
-自動で挿入される名前とコロンの直後に指摘分類をa～iで書く。
-※レビュー日時を書く場合はコロンの直後に*を書く。</v>
-      </c>
-    </row>
-    <row r="16" spans="1:21" ht="40.5" x14ac:dyDescent="0.15">
-      <c r="A16" s="272" t="s">
-        <v>38</v>
-      </c>
-      <c r="B16" s="297" t="s">
-        <v>312</v>
-      </c>
-      <c r="C16" s="272" t="s">
-        <v>308</v>
-      </c>
-      <c r="D16" s="272" t="s">
-        <v>313</v>
-      </c>
-      <c r="E16" s="298" t="s">
-        <v>314</v>
-      </c>
-      <c r="F16" s="271"/>
-      <c r="G16" s="271"/>
-      <c r="H16" s="271"/>
-      <c r="I16" s="271"/>
-      <c r="J16" s="271"/>
-      <c r="K16" s="272" t="s">
-        <v>311</v>
-      </c>
-      <c r="L16" s="295">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="M16" s="295">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="N16" s="295">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="O16" s="295">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="P16" s="295">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Q16" s="295">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R16" s="295">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="S16" s="295">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="T16" s="295">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="U16" s="296" t="str">
-        <f>IF(E16&lt;&gt;"",E16,"")</f>
-        <v>対応内容の例。
----
-対応内容はデリミタ（---）の後に記入する。</v>
-      </c>
-    </row>
-    <row r="17" spans="1:21" ht="67.5" x14ac:dyDescent="0.15">
-      <c r="A17" s="272" t="s">
-        <v>38</v>
-      </c>
-      <c r="B17" s="297" t="s">
-        <v>315</v>
-      </c>
-      <c r="C17" s="272" t="s">
-        <v>308</v>
-      </c>
-      <c r="D17" s="272" t="s">
-        <v>316</v>
-      </c>
-      <c r="E17" s="298" t="s">
-        <v>317</v>
-      </c>
-      <c r="F17" s="271"/>
-      <c r="G17" s="271"/>
-      <c r="H17" s="271"/>
-      <c r="I17" s="271"/>
-      <c r="J17" s="271"/>
-      <c r="K17" s="272" t="s">
-        <v>318</v>
-      </c>
-      <c r="L17" s="295">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="M17" s="295">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="N17" s="295">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="O17" s="295">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="P17" s="295">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Q17" s="295">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R17" s="295">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="S17" s="295">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="T17" s="295">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="U17" s="296" t="str">
-        <f>IF(E17&lt;&gt;"",E17,"")</f>
-        <v>対応内容を確認し、指摘をクローズする例。
----
-最後の行に「済」と書くと指摘をクローズできる。
-「済」の前にスペースを空けて確認日と確認者を書くこともできる。
-08/02山田 済</v>
-      </c>
-    </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.15">
-      <c r="A18" s="272"/>
-      <c r="B18" s="272"/>
-      <c r="C18" s="272"/>
-      <c r="D18" s="272"/>
-      <c r="E18" s="271"/>
-      <c r="F18" s="271"/>
-      <c r="G18" s="271"/>
-      <c r="H18" s="271"/>
-      <c r="I18" s="271"/>
-      <c r="J18" s="271"/>
-      <c r="K18" s="272"/>
-      <c r="L18" s="295">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="M18" s="295">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="N18" s="295">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="O18" s="295">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="P18" s="295">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Q18" s="295">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R18" s="295">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="S18" s="295">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="T18" s="295">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="U18" s="296" t="str">
-        <f>IF(E18&lt;&gt;"",E18,"")</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="E15:J15"/>
-    <mergeCell ref="E16:J16"/>
-    <mergeCell ref="E17:J17"/>
-    <mergeCell ref="E18:J18"/>
-  </mergeCells>
-  <phoneticPr fontId="10"/>
-  <conditionalFormatting sqref="A15:T18">
-    <cfRule type="expression" dxfId="0" priority="1" stopIfTrue="1">
-      <formula>$K15="済"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K15:K18" xr:uid="{0214427A-61DD-4497-B880-251F02694B53}">
-      <formula1>"未,済"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <hyperlinks>
-    <hyperlink ref="B15" location="'2. WA1020101(プロジェクト登録画面)'!$B$5" display="'2. WA1020101(プロジェクト登録画面)'!$B$5" xr:uid="{4FCAEF63-DC2A-422B-901A-8E67979BBD44}"/>
-    <hyperlink ref="B16" location="'2. WA1020101(プロジェクト登録画面)'!$E$60" display="'2. WA1020101(プロジェクト登録画面)'!$E$60" xr:uid="{9CA08647-9FEA-421D-BAB9-31A4D62ECF29}"/>
-    <hyperlink ref="B17" location="'2. WA1020101(プロジェクト登録画面)'!$E$62" display="'2. WA1020101(プロジェクト登録画面)'!$E$62" xr:uid="{C67B87D5-321E-476C-89E6-E4AE8A9AC757}"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.51200000000000001" footer="0.51200000000000001"/>
-  <pageSetup paperSize="9" scale="86" orientation="landscape" verticalDpi="200" r:id="rId1"/>
-  <headerFooter alignWithMargins="0"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet3">
     <pageSetUpPr fitToPage="1"/>
@@ -4545,7 +3304,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2">
     <pageSetUpPr fitToPage="1"/>
@@ -6106,7 +4865,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet4">
     <pageSetUpPr fitToPage="1"/>
@@ -6852,7 +5611,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr codeName="Sheet5">
     <pageSetUpPr fitToPage="1"/>
@@ -7358,7 +6117,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr codeName="Sheet7">
     <pageSetUpPr fitToPage="1"/>
@@ -11659,7 +10418,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr codeName="Sheet8">
     <pageSetUpPr fitToPage="1"/>
@@ -15178,7 +13937,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
@@ -16350,7 +15109,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <sheetPr codeName="Sheet6">
     <pageSetUpPr fitToPage="1"/>

</xml_diff>